<commit_message>
Stop with a clear message on unrecognised columns, handle BOM headers, add --raw-dir; 14 tests
</commit_message>
<xml_diff>
--- a/output/Sales_Report.xlsx
+++ b/output/Sales_Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Adnan Desktop\Finance\sales-data-cleaning-automation\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Adnan Desktop\Finance\sales-data-etl-pipeline\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6340D9-720B-41B2-BDFA-1A1AE0365FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA6AB73-CE46-4303-ABD8-3AA7E90A54D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -5627,7 +5627,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B4F8-4961-823B-B70C9947C830}"/>
+              <c16:uniqueId val="{00000000-97DE-4FBE-B1F5-15BA1ED18525}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5841,7 +5841,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-09AD-4304-8D52-6EA3FE1977F9}"/>
+              <c16:uniqueId val="{00000000-8225-4FFE-81C0-C48FC828606B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>